<commit_message>
Ship updated Gantt, Task List, and Resource Load builds
Pull latest packages from GitHub: Gantt 1.8.1.0 (Color by), Task List
1.0.1.0 (Norwegian RAG), and Resource Load field-binding fix, including
matching hidden white-label downloads.

Co-authored-by: JonasL <Prez0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/TaskListSampleData.xlsx
+++ b/public/downloads/TaskListSampleData.xlsx
@@ -19,16 +19,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -51,9 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -436,52 +432,52 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>RAG</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Project lead</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Start date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Estimated end</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Next milestone</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Obstacles</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -511,10 +507,10 @@
       <c r="E2" t="n">
         <v>72</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="1" t="n">
         <v>46184</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="1" t="n">
         <v>46284</v>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,10 +549,10 @@
       <c r="E3" t="n">
         <v>45</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="1" t="n">
         <v>46154</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="1" t="n">
         <v>46264</v>
       </c>
       <c r="H3" t="inlineStr">
@@ -599,10 +595,10 @@
       <c r="E4" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
         <v>46214</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>46254</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -629,7 +625,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>On track</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -645,10 +641,10 @@
       <c r="E5" t="n">
         <v>88</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="1" t="n">
         <v>46124</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -657,11 +653,7 @@
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Near release</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -671,7 +663,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>At risk</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -687,10 +679,10 @@
       <c r="E6" t="n">
         <v>55</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>46249</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -713,7 +705,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -729,10 +721,10 @@
       <c r="E7" t="n">
         <v>12</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
         <v>46249</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>46424</v>
       </c>
       <c r="H7" t="inlineStr">
@@ -755,7 +747,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>G</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -771,10 +763,10 @@
       <c r="E8" t="n">
         <v>100</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="1" t="n">
         <v>45844</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H8" t="inlineStr">
@@ -797,7 +789,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>Yellow</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -813,10 +805,10 @@
       <c r="E9" t="n">
         <v>33</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="1" t="n">
         <v>46199</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="1" t="n">
         <v>46334</v>
       </c>
       <c r="H9" t="inlineStr">

</xml_diff>